<commit_message>
feat: ensure distinct 300 test case datasets for Selenium, Security & Vulnerability, and Appium reports
</commit_message>
<xml_diff>
--- a/automation/reports/Excel/Automation_Test_Report.xlsx
+++ b/automation/reports/Excel/Automation_Test_Report.xlsx
@@ -1922,7 +1922,7 @@
     <t>Total Duration (ms)</t>
   </si>
   <si>
-    <t>4870</t>
+    <t>4991</t>
   </si>
   <si>
     <t>Defect ID</t>
@@ -2049,7 +2049,7 @@
         <v>10</v>
       </c>
       <c r="F2" t="n" s="0">
-        <v>30.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="3">
@@ -2069,7 +2069,7 @@
         <v>10</v>
       </c>
       <c r="F3" t="n" s="0">
-        <v>14.0</v>
+        <v>29.0</v>
       </c>
     </row>
     <row r="4">
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="F7" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="8">
@@ -2169,7 +2169,7 @@
         <v>10</v>
       </c>
       <c r="F8" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="9">
@@ -2209,7 +2209,7 @@
         <v>10</v>
       </c>
       <c r="F10" t="n" s="0">
-        <v>20.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="11">
@@ -2229,7 +2229,7 @@
         <v>10</v>
       </c>
       <c r="F11" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="12">
@@ -2249,7 +2249,7 @@
         <v>10</v>
       </c>
       <c r="F12" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="13">
@@ -2269,7 +2269,7 @@
         <v>10</v>
       </c>
       <c r="F13" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="14">
@@ -2289,7 +2289,7 @@
         <v>10</v>
       </c>
       <c r="F14" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="15">
@@ -2309,7 +2309,7 @@
         <v>10</v>
       </c>
       <c r="F15" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="16">
@@ -2329,7 +2329,7 @@
         <v>10</v>
       </c>
       <c r="F16" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="17">
@@ -2389,7 +2389,7 @@
         <v>10</v>
       </c>
       <c r="F19" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="20">
@@ -2429,7 +2429,7 @@
         <v>10</v>
       </c>
       <c r="F21" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="22">
@@ -2469,7 +2469,7 @@
         <v>10</v>
       </c>
       <c r="F23" t="n" s="0">
-        <v>17.0</v>
+        <v>13.0</v>
       </c>
     </row>
     <row r="24">
@@ -2489,7 +2489,7 @@
         <v>10</v>
       </c>
       <c r="F24" t="n" s="0">
-        <v>16.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="25">
@@ -2509,7 +2509,7 @@
         <v>10</v>
       </c>
       <c r="F25" t="n" s="0">
-        <v>11.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="26">
@@ -2529,7 +2529,7 @@
         <v>10</v>
       </c>
       <c r="F26" t="n" s="0">
-        <v>15.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="27">
@@ -2549,7 +2549,7 @@
         <v>10</v>
       </c>
       <c r="F27" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="28">
@@ -2589,7 +2589,7 @@
         <v>10</v>
       </c>
       <c r="F29" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="30">
@@ -2609,7 +2609,7 @@
         <v>10</v>
       </c>
       <c r="F30" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="31">
@@ -2629,7 +2629,7 @@
         <v>10</v>
       </c>
       <c r="F31" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="32">
@@ -2669,7 +2669,7 @@
         <v>10</v>
       </c>
       <c r="F33" t="n" s="0">
-        <v>15.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="34">
@@ -2689,7 +2689,7 @@
         <v>10</v>
       </c>
       <c r="F34" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="35">
@@ -2729,7 +2729,7 @@
         <v>10</v>
       </c>
       <c r="F36" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="37">
@@ -2749,7 +2749,7 @@
         <v>10</v>
       </c>
       <c r="F37" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="38">
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="F38" t="n" s="0">
-        <v>14.0</v>
+        <v>21.0</v>
       </c>
     </row>
     <row r="39">
@@ -2789,7 +2789,7 @@
         <v>10</v>
       </c>
       <c r="F39" t="n" s="0">
-        <v>14.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="40">
@@ -2809,7 +2809,7 @@
         <v>10</v>
       </c>
       <c r="F40" t="n" s="0">
-        <v>21.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="41">
@@ -2829,7 +2829,7 @@
         <v>10</v>
       </c>
       <c r="F41" t="n" s="0">
-        <v>26.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="42">
@@ -2849,7 +2849,7 @@
         <v>10</v>
       </c>
       <c r="F42" t="n" s="0">
-        <v>16.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="43">
@@ -2869,7 +2869,7 @@
         <v>10</v>
       </c>
       <c r="F43" t="n" s="0">
-        <v>18.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="44">
@@ -2889,7 +2889,7 @@
         <v>10</v>
       </c>
       <c r="F44" t="n" s="0">
-        <v>21.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="45">
@@ -2909,7 +2909,7 @@
         <v>10</v>
       </c>
       <c r="F45" t="n" s="0">
-        <v>25.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="46">
@@ -2949,7 +2949,7 @@
         <v>10</v>
       </c>
       <c r="F47" t="n" s="0">
-        <v>17.0</v>
+        <v>23.0</v>
       </c>
     </row>
     <row r="48">
@@ -2969,7 +2969,7 @@
         <v>10</v>
       </c>
       <c r="F48" t="n" s="0">
-        <v>16.0</v>
+        <v>27.0</v>
       </c>
     </row>
     <row r="49">
@@ -2989,7 +2989,7 @@
         <v>10</v>
       </c>
       <c r="F49" t="n" s="0">
-        <v>16.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="50">
@@ -3009,7 +3009,7 @@
         <v>10</v>
       </c>
       <c r="F50" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="51">
@@ -3029,7 +3029,7 @@
         <v>10</v>
       </c>
       <c r="F51" t="n" s="0">
-        <v>16.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="52">
@@ -3089,7 +3089,7 @@
         <v>10</v>
       </c>
       <c r="F54" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="55">
@@ -3109,7 +3109,7 @@
         <v>10</v>
       </c>
       <c r="F55" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="56">
@@ -3129,7 +3129,7 @@
         <v>10</v>
       </c>
       <c r="F56" t="n" s="0">
-        <v>16.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="57">
@@ -3149,7 +3149,7 @@
         <v>10</v>
       </c>
       <c r="F57" t="n" s="0">
-        <v>15.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="58">
@@ -3169,7 +3169,7 @@
         <v>10</v>
       </c>
       <c r="F58" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="59">
@@ -3209,7 +3209,7 @@
         <v>10</v>
       </c>
       <c r="F60" t="n" s="0">
-        <v>15.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="61">
@@ -3229,7 +3229,7 @@
         <v>10</v>
       </c>
       <c r="F61" t="n" s="0">
-        <v>17.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="62">
@@ -3249,7 +3249,7 @@
         <v>10</v>
       </c>
       <c r="F62" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="63">
@@ -3269,7 +3269,7 @@
         <v>10</v>
       </c>
       <c r="F63" t="n" s="0">
-        <v>19.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="64">
@@ -3289,7 +3289,7 @@
         <v>10</v>
       </c>
       <c r="F64" t="n" s="0">
-        <v>16.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="65">
@@ -3309,7 +3309,7 @@
         <v>10</v>
       </c>
       <c r="F65" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="66">
@@ -3329,7 +3329,7 @@
         <v>10</v>
       </c>
       <c r="F66" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="67">
@@ -3349,7 +3349,7 @@
         <v>10</v>
       </c>
       <c r="F67" t="n" s="0">
-        <v>16.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="68">
@@ -3369,7 +3369,7 @@
         <v>10</v>
       </c>
       <c r="F68" t="n" s="0">
-        <v>23.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="69">
@@ -3389,7 +3389,7 @@
         <v>10</v>
       </c>
       <c r="F69" t="n" s="0">
-        <v>12.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="70">
@@ -3409,7 +3409,7 @@
         <v>10</v>
       </c>
       <c r="F70" t="n" s="0">
-        <v>15.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="71">
@@ -3429,7 +3429,7 @@
         <v>10</v>
       </c>
       <c r="F71" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="72">
@@ -3449,7 +3449,7 @@
         <v>10</v>
       </c>
       <c r="F72" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="73">
@@ -3489,7 +3489,7 @@
         <v>10</v>
       </c>
       <c r="F74" t="n" s="0">
-        <v>15.0</v>
+        <v>20.0</v>
       </c>
     </row>
     <row r="75">
@@ -3509,7 +3509,7 @@
         <v>10</v>
       </c>
       <c r="F75" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="76">
@@ -3529,7 +3529,7 @@
         <v>10</v>
       </c>
       <c r="F76" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="77">
@@ -3549,7 +3549,7 @@
         <v>10</v>
       </c>
       <c r="F77" t="n" s="0">
-        <v>15.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="78">
@@ -3569,7 +3569,7 @@
         <v>10</v>
       </c>
       <c r="F78" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="79">
@@ -3589,7 +3589,7 @@
         <v>10</v>
       </c>
       <c r="F79" t="n" s="0">
-        <v>16.0</v>
+        <v>20.0</v>
       </c>
     </row>
     <row r="80">
@@ -3609,7 +3609,7 @@
         <v>10</v>
       </c>
       <c r="F80" t="n" s="0">
-        <v>19.0</v>
+        <v>12.0</v>
       </c>
     </row>
     <row r="81">
@@ -3649,7 +3649,7 @@
         <v>10</v>
       </c>
       <c r="F82" t="n" s="0">
-        <v>19.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="83">
@@ -3669,7 +3669,7 @@
         <v>10</v>
       </c>
       <c r="F83" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="84">
@@ -3689,7 +3689,7 @@
         <v>10</v>
       </c>
       <c r="F84" t="n" s="0">
-        <v>15.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="85">
@@ -3709,7 +3709,7 @@
         <v>10</v>
       </c>
       <c r="F85" t="n" s="0">
-        <v>17.0</v>
+        <v>21.0</v>
       </c>
     </row>
     <row r="86">
@@ -3729,7 +3729,7 @@
         <v>10</v>
       </c>
       <c r="F86" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="87">
@@ -3749,7 +3749,7 @@
         <v>10</v>
       </c>
       <c r="F87" t="n" s="0">
-        <v>18.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="88">
@@ -3809,7 +3809,7 @@
         <v>10</v>
       </c>
       <c r="F90" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="91">
@@ -3849,7 +3849,7 @@
         <v>10</v>
       </c>
       <c r="F92" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="93">
@@ -3869,7 +3869,7 @@
         <v>10</v>
       </c>
       <c r="F93" t="n" s="0">
-        <v>15.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="94">
@@ -3909,7 +3909,7 @@
         <v>10</v>
       </c>
       <c r="F95" t="n" s="0">
-        <v>19.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="96">
@@ -3929,7 +3929,7 @@
         <v>10</v>
       </c>
       <c r="F96" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="97">
@@ -3949,7 +3949,7 @@
         <v>10</v>
       </c>
       <c r="F97" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="98">
@@ -3989,7 +3989,7 @@
         <v>10</v>
       </c>
       <c r="F99" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="100">
@@ -4009,7 +4009,7 @@
         <v>10</v>
       </c>
       <c r="F100" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="101">
@@ -4109,7 +4109,7 @@
         <v>10</v>
       </c>
       <c r="F105" t="n" s="0">
-        <v>18.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="106">
@@ -4149,7 +4149,7 @@
         <v>10</v>
       </c>
       <c r="F107" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="108">
@@ -4169,7 +4169,7 @@
         <v>10</v>
       </c>
       <c r="F108" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="109">
@@ -4189,7 +4189,7 @@
         <v>10</v>
       </c>
       <c r="F109" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="110">
@@ -4229,7 +4229,7 @@
         <v>10</v>
       </c>
       <c r="F111" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="112">
@@ -4249,7 +4249,7 @@
         <v>10</v>
       </c>
       <c r="F112" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="113">
@@ -4269,7 +4269,7 @@
         <v>10</v>
       </c>
       <c r="F113" t="n" s="0">
-        <v>18.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="114">
@@ -4289,7 +4289,7 @@
         <v>10</v>
       </c>
       <c r="F114" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="115">
@@ -4309,7 +4309,7 @@
         <v>10</v>
       </c>
       <c r="F115" t="n" s="0">
-        <v>18.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="116">
@@ -4329,7 +4329,7 @@
         <v>10</v>
       </c>
       <c r="F116" t="n" s="0">
-        <v>16.0</v>
+        <v>22.0</v>
       </c>
     </row>
     <row r="117">
@@ -4349,7 +4349,7 @@
         <v>10</v>
       </c>
       <c r="F117" t="n" s="0">
-        <v>18.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="118">
@@ -4369,7 +4369,7 @@
         <v>10</v>
       </c>
       <c r="F118" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="119">
@@ -4389,7 +4389,7 @@
         <v>10</v>
       </c>
       <c r="F119" t="n" s="0">
-        <v>18.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="120">
@@ -4429,7 +4429,7 @@
         <v>10</v>
       </c>
       <c r="F121" t="n" s="0">
-        <v>16.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="122">
@@ -4449,7 +4449,7 @@
         <v>10</v>
       </c>
       <c r="F122" t="n" s="0">
-        <v>17.0</v>
+        <v>24.0</v>
       </c>
     </row>
     <row r="123">
@@ -4469,7 +4469,7 @@
         <v>10</v>
       </c>
       <c r="F123" t="n" s="0">
-        <v>17.0</v>
+        <v>24.0</v>
       </c>
     </row>
     <row r="124">
@@ -4489,7 +4489,7 @@
         <v>10</v>
       </c>
       <c r="F124" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="125">
@@ -4509,7 +4509,7 @@
         <v>10</v>
       </c>
       <c r="F125" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="126">
@@ -4529,7 +4529,7 @@
         <v>10</v>
       </c>
       <c r="F126" t="n" s="0">
-        <v>13.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="127">
@@ -4549,7 +4549,7 @@
         <v>10</v>
       </c>
       <c r="F127" t="n" s="0">
-        <v>17.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="128">
@@ -4569,7 +4569,7 @@
         <v>10</v>
       </c>
       <c r="F128" t="n" s="0">
-        <v>18.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="129">
@@ -4589,7 +4589,7 @@
         <v>10</v>
       </c>
       <c r="F129" t="n" s="0">
-        <v>15.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="130">
@@ -4629,7 +4629,7 @@
         <v>10</v>
       </c>
       <c r="F131" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="132">
@@ -4649,7 +4649,7 @@
         <v>10</v>
       </c>
       <c r="F132" t="n" s="0">
-        <v>14.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="133">
@@ -4669,7 +4669,7 @@
         <v>10</v>
       </c>
       <c r="F133" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="134">
@@ -4689,7 +4689,7 @@
         <v>10</v>
       </c>
       <c r="F134" t="n" s="0">
-        <v>14.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="135">
@@ -4709,7 +4709,7 @@
         <v>10</v>
       </c>
       <c r="F135" t="n" s="0">
-        <v>19.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="136">
@@ -4729,7 +4729,7 @@
         <v>10</v>
       </c>
       <c r="F136" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="137">
@@ -4769,7 +4769,7 @@
         <v>10</v>
       </c>
       <c r="F138" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="139">
@@ -4789,7 +4789,7 @@
         <v>10</v>
       </c>
       <c r="F139" t="n" s="0">
-        <v>17.0</v>
+        <v>21.0</v>
       </c>
     </row>
     <row r="140">
@@ -4809,7 +4809,7 @@
         <v>10</v>
       </c>
       <c r="F140" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="141">
@@ -4829,7 +4829,7 @@
         <v>10</v>
       </c>
       <c r="F141" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="142">
@@ -4849,7 +4849,7 @@
         <v>10</v>
       </c>
       <c r="F142" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="143">
@@ -4869,7 +4869,7 @@
         <v>10</v>
       </c>
       <c r="F143" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="144">
@@ -4889,7 +4889,7 @@
         <v>10</v>
       </c>
       <c r="F144" t="n" s="0">
-        <v>17.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="145">
@@ -4909,7 +4909,7 @@
         <v>10</v>
       </c>
       <c r="F145" t="n" s="0">
-        <v>16.0</v>
+        <v>22.0</v>
       </c>
     </row>
     <row r="146">
@@ -4929,7 +4929,7 @@
         <v>10</v>
       </c>
       <c r="F146" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="147">
@@ -4949,7 +4949,7 @@
         <v>10</v>
       </c>
       <c r="F147" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="148">
@@ -4969,7 +4969,7 @@
         <v>10</v>
       </c>
       <c r="F148" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="149">
@@ -4989,7 +4989,7 @@
         <v>10</v>
       </c>
       <c r="F149" t="n" s="0">
-        <v>15.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="150">
@@ -5009,7 +5009,7 @@
         <v>10</v>
       </c>
       <c r="F150" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="151">
@@ -5029,7 +5029,7 @@
         <v>10</v>
       </c>
       <c r="F151" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="152">
@@ -5049,7 +5049,7 @@
         <v>10</v>
       </c>
       <c r="F152" t="n" s="0">
-        <v>15.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="153">
@@ -5069,7 +5069,7 @@
         <v>10</v>
       </c>
       <c r="F153" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="154">
@@ -5089,7 +5089,7 @@
         <v>10</v>
       </c>
       <c r="F154" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="155">
@@ -5109,7 +5109,7 @@
         <v>10</v>
       </c>
       <c r="F155" t="n" s="0">
-        <v>18.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="156">
@@ -5129,7 +5129,7 @@
         <v>10</v>
       </c>
       <c r="F156" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="157">
@@ -5169,7 +5169,7 @@
         <v>10</v>
       </c>
       <c r="F158" t="n" s="0">
-        <v>17.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="159">
@@ -5189,7 +5189,7 @@
         <v>10</v>
       </c>
       <c r="F159" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="160">
@@ -5209,7 +5209,7 @@
         <v>10</v>
       </c>
       <c r="F160" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="161">
@@ -5229,7 +5229,7 @@
         <v>10</v>
       </c>
       <c r="F161" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="162">
@@ -5249,7 +5249,7 @@
         <v>10</v>
       </c>
       <c r="F162" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="163">
@@ -5269,7 +5269,7 @@
         <v>10</v>
       </c>
       <c r="F163" t="n" s="0">
-        <v>15.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="164">
@@ -5289,7 +5289,7 @@
         <v>10</v>
       </c>
       <c r="F164" t="n" s="0">
-        <v>19.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="165">
@@ -5309,7 +5309,7 @@
         <v>10</v>
       </c>
       <c r="F165" t="n" s="0">
-        <v>14.0</v>
+        <v>22.0</v>
       </c>
     </row>
     <row r="166">
@@ -5349,7 +5349,7 @@
         <v>10</v>
       </c>
       <c r="F167" t="n" s="0">
-        <v>16.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="168">
@@ -5369,7 +5369,7 @@
         <v>10</v>
       </c>
       <c r="F168" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="169">
@@ -5389,7 +5389,7 @@
         <v>10</v>
       </c>
       <c r="F169" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="170">
@@ -5409,7 +5409,7 @@
         <v>10</v>
       </c>
       <c r="F170" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="171">
@@ -5429,7 +5429,7 @@
         <v>10</v>
       </c>
       <c r="F171" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="172">
@@ -5449,7 +5449,7 @@
         <v>10</v>
       </c>
       <c r="F172" t="n" s="0">
-        <v>17.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="173">
@@ -5469,7 +5469,7 @@
         <v>10</v>
       </c>
       <c r="F173" t="n" s="0">
-        <v>16.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="174">
@@ -5489,7 +5489,7 @@
         <v>10</v>
       </c>
       <c r="F174" t="n" s="0">
-        <v>17.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="175">
@@ -5509,7 +5509,7 @@
         <v>10</v>
       </c>
       <c r="F175" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="176">
@@ -5529,7 +5529,7 @@
         <v>10</v>
       </c>
       <c r="F176" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="177">
@@ -5549,7 +5549,7 @@
         <v>10</v>
       </c>
       <c r="F177" t="n" s="0">
-        <v>15.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="178">
@@ -5569,7 +5569,7 @@
         <v>10</v>
       </c>
       <c r="F178" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="179">
@@ -5589,7 +5589,7 @@
         <v>10</v>
       </c>
       <c r="F179" t="n" s="0">
-        <v>18.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="180">
@@ -5609,7 +5609,7 @@
         <v>10</v>
       </c>
       <c r="F180" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="181">
@@ -5629,7 +5629,7 @@
         <v>10</v>
       </c>
       <c r="F181" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="182">
@@ -5649,7 +5649,7 @@
         <v>10</v>
       </c>
       <c r="F182" t="n" s="0">
-        <v>18.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="183">
@@ -5669,7 +5669,7 @@
         <v>10</v>
       </c>
       <c r="F183" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="184">
@@ -5689,7 +5689,7 @@
         <v>10</v>
       </c>
       <c r="F184" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="185">
@@ -5709,7 +5709,7 @@
         <v>10</v>
       </c>
       <c r="F185" t="n" s="0">
-        <v>15.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="186">
@@ -5769,7 +5769,7 @@
         <v>10</v>
       </c>
       <c r="F188" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="189">
@@ -5789,7 +5789,7 @@
         <v>10</v>
       </c>
       <c r="F189" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="190">
@@ -5809,7 +5809,7 @@
         <v>10</v>
       </c>
       <c r="F190" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="191">
@@ -5829,7 +5829,7 @@
         <v>10</v>
       </c>
       <c r="F191" t="n" s="0">
-        <v>18.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="192">
@@ -5869,7 +5869,7 @@
         <v>10</v>
       </c>
       <c r="F193" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="194">
@@ -5889,7 +5889,7 @@
         <v>10</v>
       </c>
       <c r="F194" t="n" s="0">
-        <v>17.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="195">
@@ -5909,7 +5909,7 @@
         <v>10</v>
       </c>
       <c r="F195" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="196">
@@ -5949,7 +5949,7 @@
         <v>10</v>
       </c>
       <c r="F197" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="198">
@@ -5969,7 +5969,7 @@
         <v>10</v>
       </c>
       <c r="F198" t="n" s="0">
-        <v>18.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="199">
@@ -5989,7 +5989,7 @@
         <v>10</v>
       </c>
       <c r="F199" t="n" s="0">
-        <v>16.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="200">
@@ -6009,7 +6009,7 @@
         <v>10</v>
       </c>
       <c r="F200" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="201">
@@ -6029,7 +6029,7 @@
         <v>10</v>
       </c>
       <c r="F201" t="n" s="0">
-        <v>17.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="202">
@@ -6049,7 +6049,7 @@
         <v>10</v>
       </c>
       <c r="F202" t="n" s="0">
-        <v>15.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="203">
@@ -6069,7 +6069,7 @@
         <v>10</v>
       </c>
       <c r="F203" t="n" s="0">
-        <v>18.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="204">
@@ -6109,7 +6109,7 @@
         <v>10</v>
       </c>
       <c r="F205" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="206">
@@ -6149,7 +6149,7 @@
         <v>10</v>
       </c>
       <c r="F207" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="208">
@@ -6169,7 +6169,7 @@
         <v>10</v>
       </c>
       <c r="F208" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="209">
@@ -6189,7 +6189,7 @@
         <v>10</v>
       </c>
       <c r="F209" t="n" s="0">
-        <v>18.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="210">
@@ -6209,7 +6209,7 @@
         <v>10</v>
       </c>
       <c r="F210" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="211">
@@ -6229,7 +6229,7 @@
         <v>10</v>
       </c>
       <c r="F211" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="212">
@@ -6249,7 +6249,7 @@
         <v>10</v>
       </c>
       <c r="F212" t="n" s="0">
-        <v>19.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="213">
@@ -6269,7 +6269,7 @@
         <v>10</v>
       </c>
       <c r="F213" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="214">
@@ -6289,7 +6289,7 @@
         <v>10</v>
       </c>
       <c r="F214" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="215">
@@ -6329,7 +6329,7 @@
         <v>10</v>
       </c>
       <c r="F216" t="n" s="0">
-        <v>14.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="217">
@@ -6349,7 +6349,7 @@
         <v>10</v>
       </c>
       <c r="F217" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="218">
@@ -6369,7 +6369,7 @@
         <v>10</v>
       </c>
       <c r="F218" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="219">
@@ -6409,7 +6409,7 @@
         <v>10</v>
       </c>
       <c r="F220" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="221">
@@ -6429,7 +6429,7 @@
         <v>10</v>
       </c>
       <c r="F221" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="222">
@@ -6449,7 +6449,7 @@
         <v>10</v>
       </c>
       <c r="F222" t="n" s="0">
-        <v>14.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="223">
@@ -6489,7 +6489,7 @@
         <v>10</v>
       </c>
       <c r="F224" t="n" s="0">
-        <v>18.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="225">
@@ -6509,7 +6509,7 @@
         <v>10</v>
       </c>
       <c r="F225" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="226">
@@ -6529,7 +6529,7 @@
         <v>10</v>
       </c>
       <c r="F226" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="227">
@@ -6549,7 +6549,7 @@
         <v>10</v>
       </c>
       <c r="F227" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="228">
@@ -6569,7 +6569,7 @@
         <v>10</v>
       </c>
       <c r="F228" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="229">
@@ -6589,7 +6589,7 @@
         <v>10</v>
       </c>
       <c r="F229" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="230">
@@ -6609,7 +6609,7 @@
         <v>10</v>
       </c>
       <c r="F230" t="n" s="0">
-        <v>18.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="231">
@@ -6629,7 +6629,7 @@
         <v>10</v>
       </c>
       <c r="F231" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="232">
@@ -6669,7 +6669,7 @@
         <v>10</v>
       </c>
       <c r="F233" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="234">
@@ -6689,7 +6689,7 @@
         <v>10</v>
       </c>
       <c r="F234" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="235">
@@ -6709,7 +6709,7 @@
         <v>10</v>
       </c>
       <c r="F235" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="236">
@@ -6749,7 +6749,7 @@
         <v>10</v>
       </c>
       <c r="F237" t="n" s="0">
-        <v>19.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="238">
@@ -6769,7 +6769,7 @@
         <v>10</v>
       </c>
       <c r="F238" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="239">
@@ -6789,7 +6789,7 @@
         <v>10</v>
       </c>
       <c r="F239" t="n" s="0">
-        <v>16.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="240">
@@ -6809,7 +6809,7 @@
         <v>10</v>
       </c>
       <c r="F240" t="n" s="0">
-        <v>15.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="241">
@@ -6829,7 +6829,7 @@
         <v>10</v>
       </c>
       <c r="F241" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="242">
@@ -6849,7 +6849,7 @@
         <v>10</v>
       </c>
       <c r="F242" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="243">
@@ -6889,7 +6889,7 @@
         <v>10</v>
       </c>
       <c r="F244" t="n" s="0">
-        <v>18.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="245">
@@ -6929,7 +6929,7 @@
         <v>10</v>
       </c>
       <c r="F246" t="n" s="0">
-        <v>15.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="247">
@@ -6969,7 +6969,7 @@
         <v>10</v>
       </c>
       <c r="F248" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="249">
@@ -7009,7 +7009,7 @@
         <v>10</v>
       </c>
       <c r="F250" t="n" s="0">
-        <v>17.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="251">
@@ -7029,7 +7029,7 @@
         <v>10</v>
       </c>
       <c r="F251" t="n" s="0">
-        <v>17.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="252">
@@ -7049,7 +7049,7 @@
         <v>10</v>
       </c>
       <c r="F252" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="253">
@@ -7089,7 +7089,7 @@
         <v>10</v>
       </c>
       <c r="F254" t="n" s="0">
-        <v>21.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="255">
@@ -7129,7 +7129,7 @@
         <v>10</v>
       </c>
       <c r="F256" t="n" s="0">
-        <v>16.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="257">
@@ -7149,7 +7149,7 @@
         <v>10</v>
       </c>
       <c r="F257" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="258">
@@ -7169,7 +7169,7 @@
         <v>10</v>
       </c>
       <c r="F258" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="259">
@@ -7189,7 +7189,7 @@
         <v>10</v>
       </c>
       <c r="F259" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="260">
@@ -7209,7 +7209,7 @@
         <v>10</v>
       </c>
       <c r="F260" t="n" s="0">
-        <v>19.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="261">
@@ -7229,7 +7229,7 @@
         <v>10</v>
       </c>
       <c r="F261" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="262">
@@ -7249,7 +7249,7 @@
         <v>10</v>
       </c>
       <c r="F262" t="n" s="0">
-        <v>17.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="263">
@@ -7269,7 +7269,7 @@
         <v>10</v>
       </c>
       <c r="F263" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="264">
@@ -7289,7 +7289,7 @@
         <v>10</v>
       </c>
       <c r="F264" t="n" s="0">
-        <v>16.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="265">
@@ -7329,7 +7329,7 @@
         <v>10</v>
       </c>
       <c r="F266" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="267">
@@ -7349,7 +7349,7 @@
         <v>10</v>
       </c>
       <c r="F267" t="n" s="0">
-        <v>18.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="268">
@@ -7389,7 +7389,7 @@
         <v>10</v>
       </c>
       <c r="F269" t="n" s="0">
-        <v>16.0</v>
+        <v>20.0</v>
       </c>
     </row>
     <row r="270">
@@ -7449,7 +7449,7 @@
         <v>10</v>
       </c>
       <c r="F272" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="273">
@@ -7469,7 +7469,7 @@
         <v>10</v>
       </c>
       <c r="F273" t="n" s="0">
-        <v>18.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="274">
@@ -7489,7 +7489,7 @@
         <v>10</v>
       </c>
       <c r="F274" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="275">
@@ -7529,7 +7529,7 @@
         <v>10</v>
       </c>
       <c r="F276" t="n" s="0">
-        <v>15.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="277">
@@ -7569,7 +7569,7 @@
         <v>10</v>
       </c>
       <c r="F278" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="279">
@@ -7609,7 +7609,7 @@
         <v>10</v>
       </c>
       <c r="F280" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="281">
@@ -7629,7 +7629,7 @@
         <v>10</v>
       </c>
       <c r="F281" t="n" s="0">
-        <v>16.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="282">
@@ -7669,7 +7669,7 @@
         <v>10</v>
       </c>
       <c r="F283" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="284">
@@ -7689,7 +7689,7 @@
         <v>10</v>
       </c>
       <c r="F284" t="n" s="0">
-        <v>16.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="285">
@@ -7729,7 +7729,7 @@
         <v>10</v>
       </c>
       <c r="F286" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="287">
@@ -7749,7 +7749,7 @@
         <v>10</v>
       </c>
       <c r="F287" t="n" s="0">
-        <v>15.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="288">
@@ -7769,7 +7769,7 @@
         <v>10</v>
       </c>
       <c r="F288" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="289">
@@ -7789,7 +7789,7 @@
         <v>10</v>
       </c>
       <c r="F289" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="290">
@@ -7809,7 +7809,7 @@
         <v>10</v>
       </c>
       <c r="F290" t="n" s="0">
-        <v>19.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="291">
@@ -7849,7 +7849,7 @@
         <v>10</v>
       </c>
       <c r="F292" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="293">
@@ -7869,7 +7869,7 @@
         <v>10</v>
       </c>
       <c r="F293" t="n" s="0">
-        <v>18.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="294">
@@ -7889,7 +7889,7 @@
         <v>10</v>
       </c>
       <c r="F294" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="295">
@@ -7909,7 +7909,7 @@
         <v>10</v>
       </c>
       <c r="F295" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="296">
@@ -7949,7 +7949,7 @@
         <v>10</v>
       </c>
       <c r="F297" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="298">
@@ -7989,7 +7989,7 @@
         <v>10</v>
       </c>
       <c r="F299" t="n" s="0">
-        <v>18.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="300">
@@ -8009,7 +8009,7 @@
         <v>10</v>
       </c>
       <c r="F300" t="n" s="0">
-        <v>15.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="301">
@@ -8029,7 +8029,7 @@
         <v>10</v>
       </c>
       <c r="F301" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
   </sheetData>
@@ -8087,7 +8087,7 @@
         <v>10</v>
       </c>
       <c r="F2" t="n" s="0">
-        <v>30.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="3">
@@ -8107,7 +8107,7 @@
         <v>10</v>
       </c>
       <c r="F3" t="n" s="0">
-        <v>14.0</v>
+        <v>29.0</v>
       </c>
     </row>
     <row r="4">
@@ -8187,7 +8187,7 @@
         <v>10</v>
       </c>
       <c r="F7" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="8">
@@ -8207,7 +8207,7 @@
         <v>10</v>
       </c>
       <c r="F8" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="9">
@@ -8247,7 +8247,7 @@
         <v>10</v>
       </c>
       <c r="F10" t="n" s="0">
-        <v>20.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="11">
@@ -8267,7 +8267,7 @@
         <v>10</v>
       </c>
       <c r="F11" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="12">
@@ -8287,7 +8287,7 @@
         <v>10</v>
       </c>
       <c r="F12" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="13">
@@ -8307,7 +8307,7 @@
         <v>10</v>
       </c>
       <c r="F13" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="14">
@@ -8327,7 +8327,7 @@
         <v>10</v>
       </c>
       <c r="F14" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="15">
@@ -8347,7 +8347,7 @@
         <v>10</v>
       </c>
       <c r="F15" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="16">
@@ -8367,7 +8367,7 @@
         <v>10</v>
       </c>
       <c r="F16" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="17">
@@ -8427,7 +8427,7 @@
         <v>10</v>
       </c>
       <c r="F19" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="20">
@@ -8467,7 +8467,7 @@
         <v>10</v>
       </c>
       <c r="F21" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="22">
@@ -8507,7 +8507,7 @@
         <v>10</v>
       </c>
       <c r="F23" t="n" s="0">
-        <v>17.0</v>
+        <v>13.0</v>
       </c>
     </row>
     <row r="24">
@@ -8527,7 +8527,7 @@
         <v>10</v>
       </c>
       <c r="F24" t="n" s="0">
-        <v>16.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="25">
@@ -8547,7 +8547,7 @@
         <v>10</v>
       </c>
       <c r="F25" t="n" s="0">
-        <v>11.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="26">
@@ -8567,7 +8567,7 @@
         <v>10</v>
       </c>
       <c r="F26" t="n" s="0">
-        <v>15.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="27">
@@ -8587,7 +8587,7 @@
         <v>10</v>
       </c>
       <c r="F27" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="28">
@@ -8627,7 +8627,7 @@
         <v>10</v>
       </c>
       <c r="F29" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="30">
@@ -8647,7 +8647,7 @@
         <v>10</v>
       </c>
       <c r="F30" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="31">
@@ -8667,7 +8667,7 @@
         <v>10</v>
       </c>
       <c r="F31" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="32">
@@ -8707,7 +8707,7 @@
         <v>10</v>
       </c>
       <c r="F33" t="n" s="0">
-        <v>15.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="34">
@@ -8727,7 +8727,7 @@
         <v>10</v>
       </c>
       <c r="F34" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="35">
@@ -8767,7 +8767,7 @@
         <v>10</v>
       </c>
       <c r="F36" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="37">
@@ -8787,7 +8787,7 @@
         <v>10</v>
       </c>
       <c r="F37" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="38">
@@ -8807,7 +8807,7 @@
         <v>10</v>
       </c>
       <c r="F38" t="n" s="0">
-        <v>14.0</v>
+        <v>21.0</v>
       </c>
     </row>
     <row r="39">
@@ -8827,7 +8827,7 @@
         <v>10</v>
       </c>
       <c r="F39" t="n" s="0">
-        <v>14.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="40">
@@ -8847,7 +8847,7 @@
         <v>10</v>
       </c>
       <c r="F40" t="n" s="0">
-        <v>21.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="41">
@@ -8867,7 +8867,7 @@
         <v>10</v>
       </c>
       <c r="F41" t="n" s="0">
-        <v>26.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="42">
@@ -8887,7 +8887,7 @@
         <v>10</v>
       </c>
       <c r="F42" t="n" s="0">
-        <v>16.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="43">
@@ -8907,7 +8907,7 @@
         <v>10</v>
       </c>
       <c r="F43" t="n" s="0">
-        <v>18.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="44">
@@ -8927,7 +8927,7 @@
         <v>10</v>
       </c>
       <c r="F44" t="n" s="0">
-        <v>21.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="45">
@@ -8947,7 +8947,7 @@
         <v>10</v>
       </c>
       <c r="F45" t="n" s="0">
-        <v>25.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="46">
@@ -8987,7 +8987,7 @@
         <v>10</v>
       </c>
       <c r="F47" t="n" s="0">
-        <v>17.0</v>
+        <v>23.0</v>
       </c>
     </row>
     <row r="48">
@@ -9007,7 +9007,7 @@
         <v>10</v>
       </c>
       <c r="F48" t="n" s="0">
-        <v>16.0</v>
+        <v>27.0</v>
       </c>
     </row>
     <row r="49">
@@ -9027,7 +9027,7 @@
         <v>10</v>
       </c>
       <c r="F49" t="n" s="0">
-        <v>16.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="50">
@@ -9047,7 +9047,7 @@
         <v>10</v>
       </c>
       <c r="F50" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="51">
@@ -9067,7 +9067,7 @@
         <v>10</v>
       </c>
       <c r="F51" t="n" s="0">
-        <v>16.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="52">
@@ -9127,7 +9127,7 @@
         <v>10</v>
       </c>
       <c r="F54" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="55">
@@ -9147,7 +9147,7 @@
         <v>10</v>
       </c>
       <c r="F55" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="56">
@@ -9167,7 +9167,7 @@
         <v>10</v>
       </c>
       <c r="F56" t="n" s="0">
-        <v>16.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="57">
@@ -9187,7 +9187,7 @@
         <v>10</v>
       </c>
       <c r="F57" t="n" s="0">
-        <v>15.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="58">
@@ -9207,7 +9207,7 @@
         <v>10</v>
       </c>
       <c r="F58" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="59">
@@ -9247,7 +9247,7 @@
         <v>10</v>
       </c>
       <c r="F60" t="n" s="0">
-        <v>15.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="61">
@@ -9267,7 +9267,7 @@
         <v>10</v>
       </c>
       <c r="F61" t="n" s="0">
-        <v>17.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="62">
@@ -9287,7 +9287,7 @@
         <v>10</v>
       </c>
       <c r="F62" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="63">
@@ -9307,7 +9307,7 @@
         <v>10</v>
       </c>
       <c r="F63" t="n" s="0">
-        <v>19.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="64">
@@ -9327,7 +9327,7 @@
         <v>10</v>
       </c>
       <c r="F64" t="n" s="0">
-        <v>16.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="65">
@@ -9347,7 +9347,7 @@
         <v>10</v>
       </c>
       <c r="F65" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="66">
@@ -9367,7 +9367,7 @@
         <v>10</v>
       </c>
       <c r="F66" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="67">
@@ -9387,7 +9387,7 @@
         <v>10</v>
       </c>
       <c r="F67" t="n" s="0">
-        <v>16.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="68">
@@ -9407,7 +9407,7 @@
         <v>10</v>
       </c>
       <c r="F68" t="n" s="0">
-        <v>23.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="69">
@@ -9427,7 +9427,7 @@
         <v>10</v>
       </c>
       <c r="F69" t="n" s="0">
-        <v>12.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="70">
@@ -9447,7 +9447,7 @@
         <v>10</v>
       </c>
       <c r="F70" t="n" s="0">
-        <v>15.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="71">
@@ -9467,7 +9467,7 @@
         <v>10</v>
       </c>
       <c r="F71" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="72">
@@ -9487,7 +9487,7 @@
         <v>10</v>
       </c>
       <c r="F72" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="73">
@@ -9527,7 +9527,7 @@
         <v>10</v>
       </c>
       <c r="F74" t="n" s="0">
-        <v>15.0</v>
+        <v>20.0</v>
       </c>
     </row>
     <row r="75">
@@ -9547,7 +9547,7 @@
         <v>10</v>
       </c>
       <c r="F75" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="76">
@@ -9567,7 +9567,7 @@
         <v>10</v>
       </c>
       <c r="F76" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="77">
@@ -9587,7 +9587,7 @@
         <v>10</v>
       </c>
       <c r="F77" t="n" s="0">
-        <v>15.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="78">
@@ -9607,7 +9607,7 @@
         <v>10</v>
       </c>
       <c r="F78" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="79">
@@ -9627,7 +9627,7 @@
         <v>10</v>
       </c>
       <c r="F79" t="n" s="0">
-        <v>16.0</v>
+        <v>20.0</v>
       </c>
     </row>
     <row r="80">
@@ -9647,7 +9647,7 @@
         <v>10</v>
       </c>
       <c r="F80" t="n" s="0">
-        <v>19.0</v>
+        <v>12.0</v>
       </c>
     </row>
     <row r="81">
@@ -9687,7 +9687,7 @@
         <v>10</v>
       </c>
       <c r="F82" t="n" s="0">
-        <v>19.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="83">
@@ -9707,7 +9707,7 @@
         <v>10</v>
       </c>
       <c r="F83" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="84">
@@ -9727,7 +9727,7 @@
         <v>10</v>
       </c>
       <c r="F84" t="n" s="0">
-        <v>15.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="85">
@@ -9747,7 +9747,7 @@
         <v>10</v>
       </c>
       <c r="F85" t="n" s="0">
-        <v>17.0</v>
+        <v>21.0</v>
       </c>
     </row>
     <row r="86">
@@ -9767,7 +9767,7 @@
         <v>10</v>
       </c>
       <c r="F86" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="87">
@@ -9787,7 +9787,7 @@
         <v>10</v>
       </c>
       <c r="F87" t="n" s="0">
-        <v>18.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="88">
@@ -9847,7 +9847,7 @@
         <v>10</v>
       </c>
       <c r="F90" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="91">
@@ -9887,7 +9887,7 @@
         <v>10</v>
       </c>
       <c r="F92" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="93">
@@ -9907,7 +9907,7 @@
         <v>10</v>
       </c>
       <c r="F93" t="n" s="0">
-        <v>15.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="94">
@@ -9947,7 +9947,7 @@
         <v>10</v>
       </c>
       <c r="F95" t="n" s="0">
-        <v>19.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="96">
@@ -9967,7 +9967,7 @@
         <v>10</v>
       </c>
       <c r="F96" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="97">
@@ -9987,7 +9987,7 @@
         <v>10</v>
       </c>
       <c r="F97" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="98">
@@ -10027,7 +10027,7 @@
         <v>10</v>
       </c>
       <c r="F99" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="100">
@@ -10047,7 +10047,7 @@
         <v>10</v>
       </c>
       <c r="F100" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="101">
@@ -10147,7 +10147,7 @@
         <v>10</v>
       </c>
       <c r="F105" t="n" s="0">
-        <v>18.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="106">
@@ -10187,7 +10187,7 @@
         <v>10</v>
       </c>
       <c r="F107" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="108">
@@ -10207,7 +10207,7 @@
         <v>10</v>
       </c>
       <c r="F108" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="109">
@@ -10227,7 +10227,7 @@
         <v>10</v>
       </c>
       <c r="F109" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="110">
@@ -10267,7 +10267,7 @@
         <v>10</v>
       </c>
       <c r="F111" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="112">
@@ -10287,7 +10287,7 @@
         <v>10</v>
       </c>
       <c r="F112" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="113">
@@ -10307,7 +10307,7 @@
         <v>10</v>
       </c>
       <c r="F113" t="n" s="0">
-        <v>18.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="114">
@@ -10327,7 +10327,7 @@
         <v>10</v>
       </c>
       <c r="F114" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="115">
@@ -10347,7 +10347,7 @@
         <v>10</v>
       </c>
       <c r="F115" t="n" s="0">
-        <v>18.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="116">
@@ -10367,7 +10367,7 @@
         <v>10</v>
       </c>
       <c r="F116" t="n" s="0">
-        <v>16.0</v>
+        <v>22.0</v>
       </c>
     </row>
     <row r="117">
@@ -10387,7 +10387,7 @@
         <v>10</v>
       </c>
       <c r="F117" t="n" s="0">
-        <v>18.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="118">
@@ -10407,7 +10407,7 @@
         <v>10</v>
       </c>
       <c r="F118" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="119">
@@ -10427,7 +10427,7 @@
         <v>10</v>
       </c>
       <c r="F119" t="n" s="0">
-        <v>18.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="120">
@@ -10467,7 +10467,7 @@
         <v>10</v>
       </c>
       <c r="F121" t="n" s="0">
-        <v>16.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="122">
@@ -10487,7 +10487,7 @@
         <v>10</v>
       </c>
       <c r="F122" t="n" s="0">
-        <v>17.0</v>
+        <v>24.0</v>
       </c>
     </row>
     <row r="123">
@@ -10507,7 +10507,7 @@
         <v>10</v>
       </c>
       <c r="F123" t="n" s="0">
-        <v>17.0</v>
+        <v>24.0</v>
       </c>
     </row>
     <row r="124">
@@ -10527,7 +10527,7 @@
         <v>10</v>
       </c>
       <c r="F124" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="125">
@@ -10547,7 +10547,7 @@
         <v>10</v>
       </c>
       <c r="F125" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="126">
@@ -10567,7 +10567,7 @@
         <v>10</v>
       </c>
       <c r="F126" t="n" s="0">
-        <v>13.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="127">
@@ -10587,7 +10587,7 @@
         <v>10</v>
       </c>
       <c r="F127" t="n" s="0">
-        <v>17.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="128">
@@ -10607,7 +10607,7 @@
         <v>10</v>
       </c>
       <c r="F128" t="n" s="0">
-        <v>18.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="129">
@@ -10627,7 +10627,7 @@
         <v>10</v>
       </c>
       <c r="F129" t="n" s="0">
-        <v>15.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="130">
@@ -10667,7 +10667,7 @@
         <v>10</v>
       </c>
       <c r="F131" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="132">
@@ -10687,7 +10687,7 @@
         <v>10</v>
       </c>
       <c r="F132" t="n" s="0">
-        <v>14.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="133">
@@ -10707,7 +10707,7 @@
         <v>10</v>
       </c>
       <c r="F133" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="134">
@@ -10727,7 +10727,7 @@
         <v>10</v>
       </c>
       <c r="F134" t="n" s="0">
-        <v>14.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="135">
@@ -10747,7 +10747,7 @@
         <v>10</v>
       </c>
       <c r="F135" t="n" s="0">
-        <v>19.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="136">
@@ -10767,7 +10767,7 @@
         <v>10</v>
       </c>
       <c r="F136" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="137">
@@ -10807,7 +10807,7 @@
         <v>10</v>
       </c>
       <c r="F138" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="139">
@@ -10827,7 +10827,7 @@
         <v>10</v>
       </c>
       <c r="F139" t="n" s="0">
-        <v>17.0</v>
+        <v>21.0</v>
       </c>
     </row>
     <row r="140">
@@ -10847,7 +10847,7 @@
         <v>10</v>
       </c>
       <c r="F140" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="141">
@@ -10867,7 +10867,7 @@
         <v>10</v>
       </c>
       <c r="F141" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="142">
@@ -10887,7 +10887,7 @@
         <v>10</v>
       </c>
       <c r="F142" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="143">
@@ -10907,7 +10907,7 @@
         <v>10</v>
       </c>
       <c r="F143" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="144">
@@ -10927,7 +10927,7 @@
         <v>10</v>
       </c>
       <c r="F144" t="n" s="0">
-        <v>17.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="145">
@@ -10947,7 +10947,7 @@
         <v>10</v>
       </c>
       <c r="F145" t="n" s="0">
-        <v>16.0</v>
+        <v>22.0</v>
       </c>
     </row>
     <row r="146">
@@ -10967,7 +10967,7 @@
         <v>10</v>
       </c>
       <c r="F146" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="147">
@@ -10987,7 +10987,7 @@
         <v>10</v>
       </c>
       <c r="F147" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="148">
@@ -11007,7 +11007,7 @@
         <v>10</v>
       </c>
       <c r="F148" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="149">
@@ -11027,7 +11027,7 @@
         <v>10</v>
       </c>
       <c r="F149" t="n" s="0">
-        <v>15.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="150">
@@ -11047,7 +11047,7 @@
         <v>10</v>
       </c>
       <c r="F150" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="151">
@@ -11067,7 +11067,7 @@
         <v>10</v>
       </c>
       <c r="F151" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="152">
@@ -11087,7 +11087,7 @@
         <v>10</v>
       </c>
       <c r="F152" t="n" s="0">
-        <v>15.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="153">
@@ -11107,7 +11107,7 @@
         <v>10</v>
       </c>
       <c r="F153" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="154">
@@ -11127,7 +11127,7 @@
         <v>10</v>
       </c>
       <c r="F154" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="155">
@@ -11147,7 +11147,7 @@
         <v>10</v>
       </c>
       <c r="F155" t="n" s="0">
-        <v>18.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="156">
@@ -11167,7 +11167,7 @@
         <v>10</v>
       </c>
       <c r="F156" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="157">
@@ -11207,7 +11207,7 @@
         <v>10</v>
       </c>
       <c r="F158" t="n" s="0">
-        <v>17.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="159">
@@ -11227,7 +11227,7 @@
         <v>10</v>
       </c>
       <c r="F159" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="160">
@@ -11247,7 +11247,7 @@
         <v>10</v>
       </c>
       <c r="F160" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="161">
@@ -11267,7 +11267,7 @@
         <v>10</v>
       </c>
       <c r="F161" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="162">
@@ -11287,7 +11287,7 @@
         <v>10</v>
       </c>
       <c r="F162" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="163">
@@ -11307,7 +11307,7 @@
         <v>10</v>
       </c>
       <c r="F163" t="n" s="0">
-        <v>15.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="164">
@@ -11327,7 +11327,7 @@
         <v>10</v>
       </c>
       <c r="F164" t="n" s="0">
-        <v>19.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="165">
@@ -11347,7 +11347,7 @@
         <v>10</v>
       </c>
       <c r="F165" t="n" s="0">
-        <v>14.0</v>
+        <v>22.0</v>
       </c>
     </row>
     <row r="166">
@@ -11387,7 +11387,7 @@
         <v>10</v>
       </c>
       <c r="F167" t="n" s="0">
-        <v>16.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="168">
@@ -11407,7 +11407,7 @@
         <v>10</v>
       </c>
       <c r="F168" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="169">
@@ -11427,7 +11427,7 @@
         <v>10</v>
       </c>
       <c r="F169" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="170">
@@ -11447,7 +11447,7 @@
         <v>10</v>
       </c>
       <c r="F170" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="171">
@@ -11467,7 +11467,7 @@
         <v>10</v>
       </c>
       <c r="F171" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="172">
@@ -11487,7 +11487,7 @@
         <v>10</v>
       </c>
       <c r="F172" t="n" s="0">
-        <v>17.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="173">
@@ -11507,7 +11507,7 @@
         <v>10</v>
       </c>
       <c r="F173" t="n" s="0">
-        <v>16.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="174">
@@ -11527,7 +11527,7 @@
         <v>10</v>
       </c>
       <c r="F174" t="n" s="0">
-        <v>17.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="175">
@@ -11547,7 +11547,7 @@
         <v>10</v>
       </c>
       <c r="F175" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="176">
@@ -11567,7 +11567,7 @@
         <v>10</v>
       </c>
       <c r="F176" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="177">
@@ -11587,7 +11587,7 @@
         <v>10</v>
       </c>
       <c r="F177" t="n" s="0">
-        <v>15.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="178">
@@ -11607,7 +11607,7 @@
         <v>10</v>
       </c>
       <c r="F178" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="179">
@@ -11627,7 +11627,7 @@
         <v>10</v>
       </c>
       <c r="F179" t="n" s="0">
-        <v>18.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="180">
@@ -11647,7 +11647,7 @@
         <v>10</v>
       </c>
       <c r="F180" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="181">
@@ -11667,7 +11667,7 @@
         <v>10</v>
       </c>
       <c r="F181" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="182">
@@ -11687,7 +11687,7 @@
         <v>10</v>
       </c>
       <c r="F182" t="n" s="0">
-        <v>18.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="183">
@@ -11707,7 +11707,7 @@
         <v>10</v>
       </c>
       <c r="F183" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="184">
@@ -11727,7 +11727,7 @@
         <v>10</v>
       </c>
       <c r="F184" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="185">
@@ -11747,7 +11747,7 @@
         <v>10</v>
       </c>
       <c r="F185" t="n" s="0">
-        <v>15.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="186">
@@ -11807,7 +11807,7 @@
         <v>10</v>
       </c>
       <c r="F188" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="189">
@@ -11827,7 +11827,7 @@
         <v>10</v>
       </c>
       <c r="F189" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="190">
@@ -11847,7 +11847,7 @@
         <v>10</v>
       </c>
       <c r="F190" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="191">
@@ -11867,7 +11867,7 @@
         <v>10</v>
       </c>
       <c r="F191" t="n" s="0">
-        <v>18.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="192">
@@ -11907,7 +11907,7 @@
         <v>10</v>
       </c>
       <c r="F193" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="194">
@@ -11927,7 +11927,7 @@
         <v>10</v>
       </c>
       <c r="F194" t="n" s="0">
-        <v>17.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="195">
@@ -11947,7 +11947,7 @@
         <v>10</v>
       </c>
       <c r="F195" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="196">
@@ -11987,7 +11987,7 @@
         <v>10</v>
       </c>
       <c r="F197" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="198">
@@ -12007,7 +12007,7 @@
         <v>10</v>
       </c>
       <c r="F198" t="n" s="0">
-        <v>18.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="199">
@@ -12027,7 +12027,7 @@
         <v>10</v>
       </c>
       <c r="F199" t="n" s="0">
-        <v>16.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="200">
@@ -12047,7 +12047,7 @@
         <v>10</v>
       </c>
       <c r="F200" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="201">
@@ -12067,7 +12067,7 @@
         <v>10</v>
       </c>
       <c r="F201" t="n" s="0">
-        <v>17.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="202">
@@ -12087,7 +12087,7 @@
         <v>10</v>
       </c>
       <c r="F202" t="n" s="0">
-        <v>15.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="203">
@@ -12107,7 +12107,7 @@
         <v>10</v>
       </c>
       <c r="F203" t="n" s="0">
-        <v>18.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="204">
@@ -12147,7 +12147,7 @@
         <v>10</v>
       </c>
       <c r="F205" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="206">
@@ -12187,7 +12187,7 @@
         <v>10</v>
       </c>
       <c r="F207" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="208">
@@ -12207,7 +12207,7 @@
         <v>10</v>
       </c>
       <c r="F208" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="209">
@@ -12227,7 +12227,7 @@
         <v>10</v>
       </c>
       <c r="F209" t="n" s="0">
-        <v>18.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="210">
@@ -12247,7 +12247,7 @@
         <v>10</v>
       </c>
       <c r="F210" t="n" s="0">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="211">
@@ -12267,7 +12267,7 @@
         <v>10</v>
       </c>
       <c r="F211" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="212">
@@ -12287,7 +12287,7 @@
         <v>10</v>
       </c>
       <c r="F212" t="n" s="0">
-        <v>19.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="213">
@@ -12307,7 +12307,7 @@
         <v>10</v>
       </c>
       <c r="F213" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="214">
@@ -12327,7 +12327,7 @@
         <v>10</v>
       </c>
       <c r="F214" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="215">
@@ -12367,7 +12367,7 @@
         <v>10</v>
       </c>
       <c r="F216" t="n" s="0">
-        <v>14.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="217">
@@ -12387,7 +12387,7 @@
         <v>10</v>
       </c>
       <c r="F217" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="218">
@@ -12407,7 +12407,7 @@
         <v>10</v>
       </c>
       <c r="F218" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="219">
@@ -12447,7 +12447,7 @@
         <v>10</v>
       </c>
       <c r="F220" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="221">
@@ -12467,7 +12467,7 @@
         <v>10</v>
       </c>
       <c r="F221" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="222">
@@ -12487,7 +12487,7 @@
         <v>10</v>
       </c>
       <c r="F222" t="n" s="0">
-        <v>14.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="223">
@@ -12527,7 +12527,7 @@
         <v>10</v>
       </c>
       <c r="F224" t="n" s="0">
-        <v>18.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="225">
@@ -12547,7 +12547,7 @@
         <v>10</v>
       </c>
       <c r="F225" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="226">
@@ -12567,7 +12567,7 @@
         <v>10</v>
       </c>
       <c r="F226" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="227">
@@ -12587,7 +12587,7 @@
         <v>10</v>
       </c>
       <c r="F227" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="228">
@@ -12607,7 +12607,7 @@
         <v>10</v>
       </c>
       <c r="F228" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="229">
@@ -12627,7 +12627,7 @@
         <v>10</v>
       </c>
       <c r="F229" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="230">
@@ -12647,7 +12647,7 @@
         <v>10</v>
       </c>
       <c r="F230" t="n" s="0">
-        <v>18.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="231">
@@ -12667,7 +12667,7 @@
         <v>10</v>
       </c>
       <c r="F231" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="232">
@@ -12707,7 +12707,7 @@
         <v>10</v>
       </c>
       <c r="F233" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="234">
@@ -12727,7 +12727,7 @@
         <v>10</v>
       </c>
       <c r="F234" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="235">
@@ -12747,7 +12747,7 @@
         <v>10</v>
       </c>
       <c r="F235" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="236">
@@ -12787,7 +12787,7 @@
         <v>10</v>
       </c>
       <c r="F237" t="n" s="0">
-        <v>19.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="238">
@@ -12807,7 +12807,7 @@
         <v>10</v>
       </c>
       <c r="F238" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="239">
@@ -12827,7 +12827,7 @@
         <v>10</v>
       </c>
       <c r="F239" t="n" s="0">
-        <v>16.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="240">
@@ -12847,7 +12847,7 @@
         <v>10</v>
       </c>
       <c r="F240" t="n" s="0">
-        <v>15.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="241">
@@ -12867,7 +12867,7 @@
         <v>10</v>
       </c>
       <c r="F241" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="242">
@@ -12887,7 +12887,7 @@
         <v>10</v>
       </c>
       <c r="F242" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="243">
@@ -12927,7 +12927,7 @@
         <v>10</v>
       </c>
       <c r="F244" t="n" s="0">
-        <v>18.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="245">
@@ -12967,7 +12967,7 @@
         <v>10</v>
       </c>
       <c r="F246" t="n" s="0">
-        <v>15.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="247">
@@ -13007,7 +13007,7 @@
         <v>10</v>
       </c>
       <c r="F248" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="249">
@@ -13047,7 +13047,7 @@
         <v>10</v>
       </c>
       <c r="F250" t="n" s="0">
-        <v>17.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="251">
@@ -13067,7 +13067,7 @@
         <v>10</v>
       </c>
       <c r="F251" t="n" s="0">
-        <v>17.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="252">
@@ -13087,7 +13087,7 @@
         <v>10</v>
       </c>
       <c r="F252" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="253">
@@ -13127,7 +13127,7 @@
         <v>10</v>
       </c>
       <c r="F254" t="n" s="0">
-        <v>21.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="255">
@@ -13167,7 +13167,7 @@
         <v>10</v>
       </c>
       <c r="F256" t="n" s="0">
-        <v>16.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="257">
@@ -13187,7 +13187,7 @@
         <v>10</v>
       </c>
       <c r="F257" t="n" s="0">
-        <v>16.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="258">
@@ -13207,7 +13207,7 @@
         <v>10</v>
       </c>
       <c r="F258" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="259">
@@ -13227,7 +13227,7 @@
         <v>10</v>
       </c>
       <c r="F259" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="260">
@@ -13247,7 +13247,7 @@
         <v>10</v>
       </c>
       <c r="F260" t="n" s="0">
-        <v>19.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="261">
@@ -13267,7 +13267,7 @@
         <v>10</v>
       </c>
       <c r="F261" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="262">
@@ -13287,7 +13287,7 @@
         <v>10</v>
       </c>
       <c r="F262" t="n" s="0">
-        <v>17.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="263">
@@ -13307,7 +13307,7 @@
         <v>10</v>
       </c>
       <c r="F263" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="264">
@@ -13327,7 +13327,7 @@
         <v>10</v>
       </c>
       <c r="F264" t="n" s="0">
-        <v>16.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="265">
@@ -13367,7 +13367,7 @@
         <v>10</v>
       </c>
       <c r="F266" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="267">
@@ -13387,7 +13387,7 @@
         <v>10</v>
       </c>
       <c r="F267" t="n" s="0">
-        <v>18.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="268">
@@ -13427,7 +13427,7 @@
         <v>10</v>
       </c>
       <c r="F269" t="n" s="0">
-        <v>16.0</v>
+        <v>20.0</v>
       </c>
     </row>
     <row r="270">
@@ -13487,7 +13487,7 @@
         <v>10</v>
       </c>
       <c r="F272" t="n" s="0">
-        <v>15.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="273">
@@ -13507,7 +13507,7 @@
         <v>10</v>
       </c>
       <c r="F273" t="n" s="0">
-        <v>18.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="274">
@@ -13527,7 +13527,7 @@
         <v>10</v>
       </c>
       <c r="F274" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="275">
@@ -13567,7 +13567,7 @@
         <v>10</v>
       </c>
       <c r="F276" t="n" s="0">
-        <v>15.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="277">
@@ -13607,7 +13607,7 @@
         <v>10</v>
       </c>
       <c r="F278" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="279">
@@ -13647,7 +13647,7 @@
         <v>10</v>
       </c>
       <c r="F280" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="281">
@@ -13667,7 +13667,7 @@
         <v>10</v>
       </c>
       <c r="F281" t="n" s="0">
-        <v>16.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="282">
@@ -13707,7 +13707,7 @@
         <v>10</v>
       </c>
       <c r="F283" t="n" s="0">
-        <v>17.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="284">
@@ -13727,7 +13727,7 @@
         <v>10</v>
       </c>
       <c r="F284" t="n" s="0">
-        <v>16.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="285">
@@ -13767,7 +13767,7 @@
         <v>10</v>
       </c>
       <c r="F286" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="287">
@@ -13787,7 +13787,7 @@
         <v>10</v>
       </c>
       <c r="F287" t="n" s="0">
-        <v>15.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="288">
@@ -13807,7 +13807,7 @@
         <v>10</v>
       </c>
       <c r="F288" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="289">
@@ -13827,7 +13827,7 @@
         <v>10</v>
       </c>
       <c r="F289" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="290">
@@ -13847,7 +13847,7 @@
         <v>10</v>
       </c>
       <c r="F290" t="n" s="0">
-        <v>19.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="291">
@@ -13887,7 +13887,7 @@
         <v>10</v>
       </c>
       <c r="F292" t="n" s="0">
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="293">
@@ -13907,7 +13907,7 @@
         <v>10</v>
       </c>
       <c r="F293" t="n" s="0">
-        <v>18.0</v>
+        <v>17.0</v>
       </c>
     </row>
     <row r="294">
@@ -13927,7 +13927,7 @@
         <v>10</v>
       </c>
       <c r="F294" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="295">
@@ -13947,7 +13947,7 @@
         <v>10</v>
       </c>
       <c r="F295" t="n" s="0">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="296">
@@ -13987,7 +13987,7 @@
         <v>10</v>
       </c>
       <c r="F297" t="n" s="0">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="298">
@@ -14027,7 +14027,7 @@
         <v>10</v>
       </c>
       <c r="F299" t="n" s="0">
-        <v>18.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="300">
@@ -14047,7 +14047,7 @@
         <v>10</v>
       </c>
       <c r="F300" t="n" s="0">
-        <v>15.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="301">
@@ -14067,7 +14067,7 @@
         <v>10</v>
       </c>
       <c r="F301" t="n" s="0">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>